<commit_message>
including new input data files that were not included in NEXTgroup's files
</commit_message>
<xml_diff>
--- a/InputData/ctrl-settings/GRA/Government Revenue Accounting.xlsx
+++ b/InputData/ctrl-settings/GRA/Government Revenue Accounting.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26327"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28526"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mmahajan\Documents\eps-us\InputData\ctrl-settings\GRA\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MeganMahajan\Documents\eps-us\InputData\ctrl-settings\GRA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2D819826-0E41-444E-85CC-5113AD7B4B57}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D2B31A74-FEF5-46AA-8455-B6AF2D8FAC31}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="17640" tabRatio="698" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="17520" tabRatio="698" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
@@ -18,7 +18,7 @@
     <sheet name="GRA-carbontax" sheetId="8" r:id="rId3"/>
     <sheet name="GRA-fueltax" sheetId="9" r:id="rId4"/>
     <sheet name="GRA-evsubsidy" sheetId="10" r:id="rId5"/>
-    <sheet name="GRA-vehbatsubsidy" sheetId="18" r:id="rId6"/>
+    <sheet name="GRA-batconsubsidy" sheetId="18" r:id="rId6"/>
     <sheet name="GRA-elecgensubsidy" sheetId="11" r:id="rId7"/>
     <sheet name="GRA-eleccapconstsubsidy" sheetId="12" r:id="rId8"/>
     <sheet name="GRA-distsolarsubsidy" sheetId="13" r:id="rId9"/>
@@ -47,26 +47,8 @@
 </workbook>
 </file>
 
-<file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
-  <authors>
-    <author>tc={4F81BCB5-E56D-426A-91DB-BCF0877CB817}</author>
-  </authors>
-  <commentList>
-    <comment ref="C15" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000001000000}">
-      <text>
-        <t>[Threaded comment]
-Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
-Comment:
-    It is recommended to leave this cell set to zero and to set a non-zero value in at least one other cell in this row.</t>
-      </text>
-    </comment>
-  </commentList>
-</comments>
-</file>
-
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="157" uniqueCount="66">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="154" uniqueCount="63">
   <si>
     <t>GRA Government Revenue Accounting</t>
   </si>
@@ -249,15 +231,6 @@
   </si>
   <si>
     <t>lever.</t>
-  </si>
-  <si>
-    <t>It is recommended that you avoid using the "deficit spending" mechanism to handle "national debt</t>
-  </si>
-  <si>
-    <t>interest" to avoid creating a feedback loop where deficit spending increases debt, which increases</t>
-  </si>
-  <si>
-    <t>interest, which further increases debt, etc.</t>
   </si>
   <si>
     <t>Corporate Taxes</t>
@@ -311,7 +284,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -339,12 +312,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="4" tint="0.59999389629810485"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -381,7 +348,7 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -401,15 +368,13 @@
 </file>
 
 <file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <person displayName="Jeffrey Rissman" id="{B752AA03-E7FD-47E9-A7F9-587DA10781FB}" userId="S::jeff@energyinnovation.onmicrosoft.com::f3f117cb-d7f5-455c-900f-329d977050a0" providerId="AD"/>
-</personList>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -447,7 +412,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -553,7 +518,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -695,23 +660,15 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
 </file>
 
-<file path=xl/threadedComments/threadedComment1.xml><?xml version="1.0" encoding="utf-8"?>
-<ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <threadedComment ref="C15" dT="2020-08-18T18:45:50.17" personId="{B752AA03-E7FD-47E9-A7F9-587DA10781FB}" id="{4F81BCB5-E56D-426A-91DB-BCF0877CB817}">
-    <text>It is recommended to leave this cell set to zero and to set a non-zero value in at least one other cell in this row.</text>
-  </threadedComment>
-</ThreadedComments>
-</file>
-
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B50"/>
+  <dimension ref="A1:B46"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="80.85546875" customWidth="1"/>
@@ -732,7 +689,7 @@
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B4" s="3" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
@@ -930,21 +887,6 @@
     <row r="46" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>60</v>
-      </c>
-    </row>
-    <row r="48" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A48" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="49" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A49" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="50" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A50" t="s">
-        <v>63</v>
       </c>
     </row>
   </sheetData>
@@ -1007,7 +949,7 @@
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="B6">
         <v>0</v>
@@ -1072,7 +1014,7 @@
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="B6">
         <v>0</v>
@@ -1108,7 +1050,7 @@
       </c>
       <c r="B2">
         <f t="array" ref="B2:B6">TRANSPOSE('Set Values Here'!B15:F15)</f>
-        <v>5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
@@ -1116,7 +1058,7 @@
         <v>48</v>
       </c>
       <c r="B3">
-        <v>0</v>
+        <v>5</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
@@ -1124,7 +1066,7 @@
         <v>49</v>
       </c>
       <c r="B4">
-        <v>5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
@@ -1137,7 +1079,7 @@
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="B6">
         <v>0</v>
@@ -1173,7 +1115,7 @@
       </c>
       <c r="B2">
         <f t="array" ref="B2:B6">TRANSPOSE('Set Values Here'!B16:F16)</f>
-        <v>5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
@@ -1189,7 +1131,7 @@
         <v>49</v>
       </c>
       <c r="B4">
-        <v>5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
@@ -1202,7 +1144,7 @@
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="B6">
         <v>0</v>
@@ -1214,7 +1156,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <sheetPr>
     <tabColor rgb="FF92D050"/>
   </sheetPr>
@@ -1272,7 +1214,7 @@
         <v>50</v>
       </c>
       <c r="F7" s="7" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
@@ -1312,7 +1254,7 @@
         <v>0</v>
       </c>
       <c r="F9">
-        <v>5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
@@ -1420,13 +1362,13 @@
         <v>42</v>
       </c>
       <c r="B15">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="C15" s="14">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D15">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="E15">
         <v>0</v>
@@ -1440,13 +1382,13 @@
         <v>34</v>
       </c>
       <c r="B16">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="C16">
         <v>5</v>
       </c>
       <c r="D16">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="E16">
         <v>0</v>
@@ -1487,7 +1429,7 @@
         <v>50</v>
       </c>
       <c r="F21" s="7" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.25">
@@ -1525,7 +1467,7 @@
       </c>
       <c r="C23" s="10">
         <f t="shared" si="1"/>
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="D23" s="10">
         <f t="shared" si="1"/>
@@ -1537,7 +1479,7 @@
       </c>
       <c r="F23" s="10">
         <f t="shared" si="1"/>
-        <v>0.5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.25">
@@ -1671,15 +1613,15 @@
       </c>
       <c r="B29" s="10">
         <f t="shared" ref="B29:F29" si="7">IFERROR(B15/SUM($B15:$F15),1/COUNT($B15:$F15))</f>
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="C29" s="10">
         <f t="shared" si="7"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D29" s="10">
         <f t="shared" si="7"/>
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="E29" s="10">
         <f t="shared" si="7"/>
@@ -1696,15 +1638,15 @@
       </c>
       <c r="B30" s="10">
         <f t="shared" ref="B30:F30" si="8">IFERROR(B16/SUM($B16:$F16),1/COUNT($B16:$F16))</f>
-        <v>0.33333333333333331</v>
+        <v>0</v>
       </c>
       <c r="C30" s="10">
         <f t="shared" si="8"/>
-        <v>0.33333333333333331</v>
+        <v>1</v>
       </c>
       <c r="D30" s="10">
         <f t="shared" si="8"/>
-        <v>0.33333333333333331</v>
+        <v>0</v>
       </c>
       <c r="E30" s="10">
         <f t="shared" si="8"/>
@@ -1718,7 +1660,6 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
-  <legacyDrawing r:id="rId2"/>
 </worksheet>
 </file>
 
@@ -1776,7 +1717,7 @@
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="B6">
         <v>0</v>
@@ -1841,10 +1782,10 @@
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="B6">
-        <v>5</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -1906,7 +1847,7 @@
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="B6">
         <v>0</v>
@@ -1971,7 +1912,7 @@
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="B6">
         <v>0</v>
@@ -2036,7 +1977,7 @@
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="B6">
         <v>0</v>
@@ -2101,7 +2042,7 @@
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="B6">
         <v>0</v>
@@ -2166,7 +2107,7 @@
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="B6">
         <v>0</v>
@@ -2175,175 +2116,4 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
-</file>
-
-<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100E59C87379D9A4242BB3A95F198D6F941" ma:contentTypeVersion="4" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="07a235b40ffe2d9a960bde50f6511605">
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="40f4d404-d193-41dc-bb72-733c1e774208" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="485fc8e6f691b86ce0aee9b7e82feca0" ns2:_="">
-    <xsd:import namespace="40f4d404-d193-41dc-bb72-733c1e774208"/>
-    <xsd:element name="properties">
-      <xsd:complexType>
-        <xsd:sequence>
-          <xsd:element name="documentManagement">
-            <xsd:complexType>
-              <xsd:all>
-                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceObjectDetectorVersions" minOccurs="0"/>
-              </xsd:all>
-            </xsd:complexType>
-          </xsd:element>
-        </xsd:sequence>
-      </xsd:complexType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="40f4d404-d193-41dc-bb72-733c1e774208" elementFormDefault="qualified">
-    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <xsd:element name="MediaServiceMetadata" ma:index="8" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceFastMetadata" ma:index="9" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceSearchProperties" ma:index="10" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceObjectDetectorVersions" ma:index="11" nillable="true" ma:displayName="MediaServiceObjectDetectorVersions" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceObjectDetectorVersions" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
-    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
-    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
-    <xsd:element name="coreProperties" type="CT_coreProperties"/>
-    <xsd:complexType name="CT_coreProperties">
-      <xsd:all>
-        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
-        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
-        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
-          <xsd:annotation>
-            <xsd:documentation>
-                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
-                    </xsd:documentation>
-          </xsd:annotation>
-        </xsd:element>
-        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-      </xsd:all>
-    </xsd:complexType>
-  </xsd:schema>
-  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
-    <xs:element name="Person">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:DisplayName" minOccurs="0"/>
-          <xs:element ref="pc:AccountId" minOccurs="0"/>
-          <xs:element ref="pc:AccountType" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="DisplayName" type="xs:string"/>
-    <xs:element name="AccountId" type="xs:string"/>
-    <xs:element name="AccountType" type="xs:string"/>
-    <xs:element name="BDCAssociatedEntity">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
-        </xs:sequence>
-        <xs:attribute ref="pc:EntityNamespace"/>
-        <xs:attribute ref="pc:EntityName"/>
-        <xs:attribute ref="pc:SystemInstanceName"/>
-        <xs:attribute ref="pc:AssociationName"/>
-      </xs:complexType>
-    </xs:element>
-    <xs:attribute name="EntityNamespace" type="xs:string"/>
-    <xs:attribute name="EntityName" type="xs:string"/>
-    <xs:attribute name="SystemInstanceName" type="xs:string"/>
-    <xs:attribute name="AssociationName" type="xs:string"/>
-    <xs:element name="BDCEntity">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
-          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
-          <xs:element ref="pc:EntityId1" minOccurs="0"/>
-          <xs:element ref="pc:EntityId2" minOccurs="0"/>
-          <xs:element ref="pc:EntityId3" minOccurs="0"/>
-          <xs:element ref="pc:EntityId4" minOccurs="0"/>
-          <xs:element ref="pc:EntityId5" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="EntityDisplayName" type="xs:string"/>
-    <xs:element name="EntityInstanceReference" type="xs:string"/>
-    <xs:element name="EntityId1" type="xs:string"/>
-    <xs:element name="EntityId2" type="xs:string"/>
-    <xs:element name="EntityId3" type="xs:string"/>
-    <xs:element name="EntityId4" type="xs:string"/>
-    <xs:element name="EntityId5" type="xs:string"/>
-    <xs:element name="Terms">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="TermInfo">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:TermName" minOccurs="0"/>
-          <xs:element ref="pc:TermId" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="TermName" type="xs:string"/>
-    <xs:element name="TermId" type="xs:string"/>
-  </xs:schema>
-</ct:contentTypeSchema>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{39E7D76A-13C4-4468-B9E7-966D6699C224}"/>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FB3639C8-F38D-4401-BBB7-3368296CDA6E}"/>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{77B6D5D2-E63B-4E4C-913E-5078D7C0DC80}"/>
 </file>
</xml_diff>

<commit_message>
updates to GRA and WebApp Data
</commit_message>
<xml_diff>
--- a/InputData/ctrl-settings/GRA/Government Revenue Accounting.xlsx
+++ b/InputData/ctrl-settings/GRA/Government Revenue Accounting.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28526"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MeganMahajan\Documents\eps-us\InputData\ctrl-settings\GRA\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Rachel Goldstein\Desktop\EPS Models\SouthKorea EPS\InputData\ctrl-settings\GRA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D2B31A74-FEF5-46AA-8455-B6AF2D8FAC31}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{712FC88C-EE7B-4B45-B6D6-5D154A3E71AA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="17520" tabRatio="698" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1548" yWindow="432" windowWidth="19536" windowHeight="13104" tabRatio="698" firstSheet="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
@@ -329,7 +329,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -348,7 +348,6 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -365,10 +364,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -669,17 +664,17 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:B46"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="80.85546875" customWidth="1"/>
+    <col min="2" max="2" width="80.88671875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
         <v>1</v>
       </c>
@@ -687,72 +682,72 @@
         <v>24</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="B4" s="3" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="B5" s="3" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A20" s="2">
         <v>1</v>
       </c>
@@ -760,7 +755,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A21" s="2">
         <v>2</v>
       </c>
@@ -768,7 +763,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A22" s="2">
         <v>3</v>
       </c>
@@ -776,7 +771,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A23" s="2">
         <v>4</v>
       </c>
@@ -784,7 +779,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A24" s="2">
         <v>5</v>
       </c>
@@ -792,99 +787,99 @@
         <v>16</v>
       </c>
     </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A26" s="4" t="s">
         <v>33</v>
       </c>
       <c r="B26" s="5"/>
     </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="32" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="35" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="37" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="38" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="39" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="41" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A41" s="12" t="s">
         <v>55</v>
       </c>
       <c r="B41" s="13"/>
     </row>
-    <row r="42" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="43" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="44" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="45" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="46" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
         <v>60</v>
       </c>
@@ -901,12 +896,12 @@
     <tabColor theme="4" tint="-0.249977111117893"/>
   </sheetPr>
   <dimension ref="A1:B6"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="34.85546875" customWidth="1"/>
+    <col min="1" max="1" width="34.88671875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" s="3" t="s">
         <v>23</v>
       </c>
@@ -914,7 +909,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>47</v>
       </c>
@@ -923,7 +918,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>48</v>
       </c>
@@ -931,7 +926,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>49</v>
       </c>
@@ -939,7 +934,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>50</v>
       </c>
@@ -947,7 +942,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>61</v>
       </c>
@@ -966,12 +961,12 @@
     <tabColor theme="4" tint="-0.249977111117893"/>
   </sheetPr>
   <dimension ref="A1:B6"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="34.85546875" customWidth="1"/>
+    <col min="1" max="1" width="34.88671875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" s="3" t="s">
         <v>23</v>
       </c>
@@ -979,7 +974,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>47</v>
       </c>
@@ -988,7 +983,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>48</v>
       </c>
@@ -996,7 +991,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>49</v>
       </c>
@@ -1004,7 +999,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>50</v>
       </c>
@@ -1012,7 +1007,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>61</v>
       </c>
@@ -1031,12 +1026,12 @@
     <tabColor theme="4" tint="-0.249977111117893"/>
   </sheetPr>
   <dimension ref="A1:B6"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="34.85546875" customWidth="1"/>
+    <col min="1" max="1" width="34.88671875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" s="3" t="s">
         <v>23</v>
       </c>
@@ -1044,7 +1039,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>47</v>
       </c>
@@ -1053,7 +1048,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>48</v>
       </c>
@@ -1061,7 +1056,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>49</v>
       </c>
@@ -1069,7 +1064,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>50</v>
       </c>
@@ -1077,7 +1072,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>61</v>
       </c>
@@ -1096,12 +1091,12 @@
     <tabColor theme="4" tint="-0.249977111117893"/>
   </sheetPr>
   <dimension ref="A1:B6"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="34.85546875" customWidth="1"/>
+    <col min="1" max="1" width="34.88671875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" s="3" t="s">
         <v>23</v>
       </c>
@@ -1109,7 +1104,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>47</v>
       </c>
@@ -1118,7 +1113,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>48</v>
       </c>
@@ -1126,7 +1121,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>49</v>
       </c>
@@ -1134,7 +1129,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>50</v>
       </c>
@@ -1142,7 +1137,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>61</v>
       </c>
@@ -1161,33 +1156,33 @@
     <tabColor rgb="FF92D050"/>
   </sheetPr>
   <dimension ref="A1:F30"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="32" customWidth="1"/>
     <col min="2" max="6" width="12" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A6" s="8" t="s">
         <v>51</v>
       </c>
@@ -1197,7 +1192,7 @@
       <c r="E6" s="9"/>
       <c r="F6" s="9"/>
     </row>
-    <row r="7" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A7" s="6" t="s">
         <v>46</v>
       </c>
@@ -1217,7 +1212,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>35</v>
       </c>
@@ -1237,7 +1232,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>36</v>
       </c>
@@ -1257,7 +1252,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>37</v>
       </c>
@@ -1277,7 +1272,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>38</v>
       </c>
@@ -1297,7 +1292,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>39</v>
       </c>
@@ -1317,7 +1312,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>40</v>
       </c>
@@ -1337,7 +1332,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>41</v>
       </c>
@@ -1357,14 +1352,14 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>42</v>
       </c>
       <c r="B15">
         <v>0</v>
       </c>
-      <c r="C15" s="14">
+      <c r="C15">
         <v>5</v>
       </c>
       <c r="D15">
@@ -1377,7 +1372,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>34</v>
       </c>
@@ -1397,7 +1392,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A19" s="12" t="s">
         <v>52</v>
       </c>
@@ -1407,12 +1402,12 @@
       <c r="E19" s="13"/>
       <c r="F19" s="13"/>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A20" s="11" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="21" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A21" s="6" t="s">
         <v>46</v>
       </c>
@@ -1432,7 +1427,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>35</v>
       </c>
@@ -1457,7 +1452,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>36</v>
       </c>
@@ -1482,7 +1477,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>37</v>
       </c>
@@ -1507,7 +1502,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>38</v>
       </c>
@@ -1532,7 +1527,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>39</v>
       </c>
@@ -1557,7 +1552,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>40</v>
       </c>
@@ -1582,7 +1577,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>41</v>
       </c>
@@ -1607,7 +1602,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>42</v>
       </c>
@@ -1632,7 +1627,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
         <v>34</v>
       </c>
@@ -1669,12 +1664,12 @@
     <tabColor theme="4" tint="-0.249977111117893"/>
   </sheetPr>
   <dimension ref="A1:B6"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="34.85546875" customWidth="1"/>
+    <col min="1" max="1" width="34.88671875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" s="3" t="s">
         <v>23</v>
       </c>
@@ -1682,7 +1677,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>47</v>
       </c>
@@ -1691,7 +1686,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>48</v>
       </c>
@@ -1699,7 +1694,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>49</v>
       </c>
@@ -1707,7 +1702,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>50</v>
       </c>
@@ -1715,7 +1710,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>61</v>
       </c>
@@ -1734,12 +1729,12 @@
     <tabColor theme="4" tint="-0.249977111117893"/>
   </sheetPr>
   <dimension ref="A1:B6"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="34.85546875" customWidth="1"/>
+    <col min="1" max="1" width="34.88671875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" s="3" t="s">
         <v>23</v>
       </c>
@@ -1747,7 +1742,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>47</v>
       </c>
@@ -1756,7 +1751,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>48</v>
       </c>
@@ -1764,7 +1759,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>49</v>
       </c>
@@ -1772,7 +1767,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>50</v>
       </c>
@@ -1780,7 +1775,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>61</v>
       </c>
@@ -1799,12 +1794,12 @@
     <tabColor theme="4" tint="-0.249977111117893"/>
   </sheetPr>
   <dimension ref="A1:B6"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="34.85546875" customWidth="1"/>
+    <col min="1" max="1" width="34.88671875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" s="3" t="s">
         <v>23</v>
       </c>
@@ -1812,7 +1807,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>47</v>
       </c>
@@ -1821,7 +1816,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>48</v>
       </c>
@@ -1829,7 +1824,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>49</v>
       </c>
@@ -1837,7 +1832,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>50</v>
       </c>
@@ -1845,7 +1840,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>61</v>
       </c>
@@ -1864,12 +1859,12 @@
     <tabColor theme="4" tint="-0.249977111117893"/>
   </sheetPr>
   <dimension ref="A1:B6"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="34.85546875" customWidth="1"/>
+    <col min="1" max="1" width="34.88671875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" s="3" t="s">
         <v>23</v>
       </c>
@@ -1877,7 +1872,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>47</v>
       </c>
@@ -1886,7 +1881,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>48</v>
       </c>
@@ -1894,7 +1889,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>49</v>
       </c>
@@ -1902,7 +1897,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>50</v>
       </c>
@@ -1910,7 +1905,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>61</v>
       </c>
@@ -1929,12 +1924,12 @@
     <tabColor theme="4" tint="-0.249977111117893"/>
   </sheetPr>
   <dimension ref="A1:B6"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="34.85546875" customWidth="1"/>
+    <col min="1" max="1" width="34.88671875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" s="3" t="s">
         <v>23</v>
       </c>
@@ -1942,7 +1937,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>47</v>
       </c>
@@ -1951,7 +1946,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>48</v>
       </c>
@@ -1959,7 +1954,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>49</v>
       </c>
@@ -1967,7 +1962,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>50</v>
       </c>
@@ -1975,7 +1970,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>61</v>
       </c>
@@ -1994,12 +1989,12 @@
     <tabColor theme="4" tint="-0.249977111117893"/>
   </sheetPr>
   <dimension ref="A1:B6"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="34.85546875" customWidth="1"/>
+    <col min="1" max="1" width="34.88671875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" s="3" t="s">
         <v>23</v>
       </c>
@@ -2007,7 +2002,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>47</v>
       </c>
@@ -2016,7 +2011,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>48</v>
       </c>
@@ -2024,7 +2019,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>49</v>
       </c>
@@ -2032,7 +2027,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>50</v>
       </c>
@@ -2040,7 +2035,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>61</v>
       </c>
@@ -2059,12 +2054,12 @@
     <tabColor theme="4" tint="-0.249977111117893"/>
   </sheetPr>
   <dimension ref="A1:B6"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="34.85546875" customWidth="1"/>
+    <col min="1" max="1" width="34.88671875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" s="3" t="s">
         <v>23</v>
       </c>
@@ -2072,7 +2067,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>47</v>
       </c>
@@ -2081,7 +2076,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>48</v>
       </c>
@@ -2089,7 +2084,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>49</v>
       </c>
@@ -2097,7 +2092,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>50</v>
       </c>
@@ -2105,7 +2100,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>61</v>
       </c>

</xml_diff>